<commit_message>
Actualiza BD y elimina antiguos EC y agrega parte 1 nuevos EC
</commit_message>
<xml_diff>
--- a/Data/EC/CC-1536905.xlsx
+++ b/Data/EC/CC-1536905.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laura Wilches\Documents\2_ Macro Comfenalco Cartagena\Macro Aviso Incumplimiento y demás\Estados De Cuenta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Operaciones\OneDrive - NIYARAKY COLOMBIA SAS OLD2\Escritorio\2- MACRO COMFENALCO CARTAGENA ACTUALIZACION\2- MACRO COMFENALCO CARTAGENA ACTUALIZACION\Estados De Cuenta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94BE2DB0-6652-43D1-86E0-74B8D107C07F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{347EFB42-230E-4467-81A0-533008114331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B3B32525-1756-440F-94EF-D4F362BF6B8E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4C69759F-9FA3-4DD0-9F80-139D6FA08831}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -500,22 +500,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>633769</xdr:colOff>
+      <xdr:colOff>717113</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>55950</xdr:rowOff>
+      <xdr:rowOff>75000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>437794</xdr:colOff>
+      <xdr:colOff>435413</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>125025</xdr:rowOff>
+      <xdr:rowOff>115500</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E93E4F4-B861-CE3A-68AA-DE825B48FAF5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{465B47D1-6490-DACD-E6F0-93758AD2BEC2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -524,7 +524,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -537,7 +537,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="890944" y="236925"/>
+          <a:off x="964763" y="265500"/>
           <a:ext cx="975600" cy="612000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -866,23 +866,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BCF6C79-FB7F-4206-A4E6-21EDF607A494}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{047A3821-23FF-42EB-B840-EAAD8B9442AA}">
   <dimension ref="B2:J30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.59765625" customWidth="1"/>
-    <col min="2" max="2" width="18.9296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.73046875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.73046875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.59765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="3"/>
       <c r="C2" s="28"/>
       <c r="D2" s="29" t="s">
@@ -895,7 +895,7 @@
       <c r="I2" s="29"/>
       <c r="J2" s="29"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" s="3"/>
       <c r="C3" s="28"/>
       <c r="D3" s="30"/>
@@ -906,7 +906,7 @@
       <c r="I3" s="30"/>
       <c r="J3" s="30"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="3"/>
       <c r="C4" s="28"/>
       <c r="D4" s="30"/>
@@ -917,7 +917,7 @@
       <c r="I4" s="30"/>
       <c r="J4" s="30"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="28"/>
       <c r="D5" s="31"/>
@@ -928,8 +928,8 @@
       <c r="I5" s="31"/>
       <c r="J5" s="31"/>
     </row>
-    <row r="6" spans="2:10" ht="9" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:10" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
@@ -944,8 +944,8 @@
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
     </row>
-    <row r="8" spans="2:10" ht="7.5" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:10" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
@@ -960,8 +960,8 @@
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
     </row>
-    <row r="10" spans="2:10" ht="6.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:10" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
         <v>23</v>
       </c>
@@ -976,8 +976,8 @@
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
     </row>
-    <row r="12" spans="2:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>24</v>
       </c>
@@ -996,7 +996,7 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>0</v>
       </c>
@@ -1025,7 +1025,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="15" t="s">
         <v>6</v>
       </c>
@@ -1048,7 +1048,7 @@
       <c r="I16" s="19"/>
       <c r="J16" s="20"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="15" t="s">
         <v>6</v>
       </c>
@@ -1071,7 +1071,7 @@
       <c r="I17" s="19"/>
       <c r="J17" s="20"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="15" t="s">
         <v>6</v>
       </c>
@@ -1094,7 +1094,7 @@
       <c r="I18" s="19"/>
       <c r="J18" s="20"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="15" t="s">
         <v>6</v>
       </c>
@@ -1117,7 +1117,7 @@
       <c r="I19" s="19"/>
       <c r="J19" s="20"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>6</v>
       </c>
@@ -1140,7 +1140,7 @@
       <c r="I20" s="19"/>
       <c r="J20" s="20"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="15" t="s">
         <v>6</v>
       </c>
@@ -1163,7 +1163,7 @@
       <c r="I21" s="19"/>
       <c r="J21" s="20"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="15" t="s">
         <v>6</v>
       </c>
@@ -1186,7 +1186,7 @@
       <c r="I22" s="19"/>
       <c r="J22" s="20"/>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="15" t="s">
         <v>6</v>
       </c>
@@ -1209,7 +1209,7 @@
       <c r="I23" s="19"/>
       <c r="J23" s="20"/>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="21" t="s">
         <v>6</v>
       </c>
@@ -1232,7 +1232,7 @@
       <c r="I24" s="25"/>
       <c r="J24" s="26"/>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="32" t="s">
         <v>30</v>
       </c>
@@ -1243,7 +1243,7 @@
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="32" t="s">
         <v>29</v>
       </c>

</xml_diff>